<commit_message>
atualização dos dados de 1Q27
</commit_message>
<xml_diff>
--- a/analise_eua/semicondutores/nvidia/nvda_indicators.xlsx
+++ b/analise_eua/semicondutores/nvidia/nvda_indicators.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,13 +49,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,163 +436,163 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>2026</v>
       </c>
       <c r="B2" t="n">
-        <v>38.78</v>
+        <v>38.77</v>
       </c>
       <c r="C2" t="n">
         <v>38.77</v>
@@ -596,7 +610,7 @@
         <v>29.59</v>
       </c>
       <c r="H2" t="n">
-        <v>4655735670</v>
+        <v>4655492080</v>
       </c>
       <c r="I2" t="n">
         <v>11412</v>
@@ -669,14 +683,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="B3" t="n">
         <v>40.44</v>
       </c>
       <c r="C3" t="n">
-        <v>40.42</v>
+        <v>40.41</v>
       </c>
       <c r="D3" t="n">
         <v>2.47</v>
@@ -691,7 +705,7 @@
         <v>37.16</v>
       </c>
       <c r="H3" t="n">
-        <v>2947582200</v>
+        <v>2947336650</v>
       </c>
       <c r="I3" t="n">
         <v>10270</v>
@@ -764,7 +778,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="B4" t="n">
@@ -859,7 +873,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>2023</v>
       </c>
       <c r="B5" t="n">
@@ -954,7 +968,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="B6" t="n">
@@ -1049,7 +1063,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="B7" t="n">
@@ -1144,7 +1158,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="B8" t="n">
@@ -1239,7 +1253,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>2019</v>
       </c>
       <c r="B9" t="n">
@@ -1334,7 +1348,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="B10" t="n">
@@ -1429,7 +1443,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="1" t="n">
         <v>2017</v>
       </c>
       <c r="B11" t="n">
@@ -1534,1583 +1548,1678 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>45956</v>
+      <c r="A2" s="2" t="n">
+        <v>46138</v>
       </c>
       <c r="B2" t="n">
-        <v>154.36</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>51.26</v>
+        <v>35.89</v>
       </c>
       <c r="D2" t="n">
-        <v>1.95</v>
+        <v>2.79</v>
       </c>
       <c r="E2" t="n">
-        <v>36761</v>
+        <v>54533</v>
       </c>
       <c r="F2" t="n">
-        <v>55.98</v>
+        <v>71.45999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>41.41</v>
+        <v>24.79</v>
       </c>
       <c r="H2" t="n">
-        <v>4925730960</v>
+        <v>4846757020</v>
       </c>
       <c r="I2" t="n">
-        <v>10822</v>
+        <v>12814</v>
       </c>
       <c r="J2" t="n">
-        <v>60608</v>
+        <v>80572</v>
       </c>
       <c r="K2" t="n">
-        <v>-49786</v>
+        <v>-67758</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.45</v>
+        <v>-0.47</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.42</v>
+        <v>-0.35</v>
       </c>
       <c r="N2" t="n">
-        <v>45.04</v>
+        <v>34.45</v>
       </c>
       <c r="O2" t="n">
-        <v>81.09</v>
+        <v>69.28</v>
       </c>
       <c r="P2" t="n">
-        <v>70.16</v>
+        <v>54.78</v>
       </c>
       <c r="Q2" t="n">
-        <v>23751</v>
+        <v>50344</v>
       </c>
       <c r="R2" t="n">
-        <v>-9024</v>
+        <v>-26429</v>
       </c>
       <c r="S2" t="n">
-        <v>-14880</v>
+        <v>-21283</v>
       </c>
       <c r="T2" t="n">
-        <v>22115</v>
+        <v>48587</v>
       </c>
       <c r="U2" t="n">
-        <v>1636</v>
+        <v>1757</v>
       </c>
       <c r="V2" t="n">
-        <v>3062</v>
+        <v>3487</v>
       </c>
       <c r="W2" t="n">
-        <v>4705</v>
+        <v>6321</v>
       </c>
       <c r="X2" t="n">
-        <v>19437</v>
+        <v>22793</v>
       </c>
       <c r="Y2" t="n">
-        <v>90417</v>
+        <v>107111</v>
       </c>
       <c r="Z2" t="n">
-        <v>31.39</v>
+        <v>15.48</v>
       </c>
       <c r="AA2" t="n">
-        <v>84223</v>
+        <v>137069</v>
       </c>
       <c r="AB2" t="n">
-        <v>78615</v>
+        <v>118131</v>
       </c>
       <c r="AC2" t="n">
         <v>0.01</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.76</v>
+        <v>0.42</v>
       </c>
       <c r="AE2" t="n">
-        <v>12456</v>
+        <v>19312</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45865</v>
+      <c r="A3" s="2" t="n">
+        <v>45956</v>
       </c>
       <c r="B3" t="n">
-        <v>164.01</v>
+        <v>154.36</v>
       </c>
       <c r="C3" t="n">
-        <v>53.57</v>
+        <v>51.26</v>
       </c>
       <c r="D3" t="n">
-        <v>1.87</v>
+        <v>1.95</v>
       </c>
       <c r="E3" t="n">
-        <v>29109</v>
+        <v>36761</v>
       </c>
       <c r="F3" t="n">
-        <v>56.53</v>
+        <v>55.98</v>
       </c>
       <c r="G3" t="n">
-        <v>43.27</v>
+        <v>41.4</v>
       </c>
       <c r="H3" t="n">
-        <v>4333493100</v>
+        <v>4925487690</v>
       </c>
       <c r="I3" t="n">
-        <v>10598</v>
+        <v>10822</v>
       </c>
       <c r="J3" t="n">
-        <v>56791</v>
+        <v>60608</v>
       </c>
       <c r="K3" t="n">
-        <v>-46193</v>
+        <v>-49786</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.5</v>
+        <v>-0.45</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.46</v>
+        <v>-0.42</v>
       </c>
       <c r="N3" t="n">
-        <v>47.21</v>
+        <v>45.04</v>
       </c>
       <c r="O3" t="n">
-        <v>81</v>
+        <v>81.09</v>
       </c>
       <c r="P3" t="n">
-        <v>69.58</v>
+        <v>70.16</v>
       </c>
       <c r="Q3" t="n">
-        <v>15365</v>
+        <v>23751</v>
       </c>
       <c r="R3" t="n">
-        <v>-7127</v>
+        <v>-9024</v>
       </c>
       <c r="S3" t="n">
-        <v>-11833</v>
+        <v>-14880</v>
       </c>
       <c r="T3" t="n">
-        <v>13470</v>
+        <v>22115</v>
       </c>
       <c r="U3" t="n">
-        <v>1895</v>
+        <v>1636</v>
       </c>
       <c r="V3" t="n">
-        <v>2721</v>
+        <v>3062</v>
       </c>
       <c r="W3" t="n">
-        <v>4291</v>
+        <v>4705</v>
       </c>
       <c r="X3" t="n">
-        <v>17481</v>
+        <v>19437</v>
       </c>
       <c r="Y3" t="n">
-        <v>77962</v>
+        <v>90417</v>
       </c>
       <c r="Z3" t="n">
-        <v>36.97</v>
+        <v>31.39</v>
       </c>
       <c r="AA3" t="n">
-        <v>66129</v>
+        <v>84223</v>
       </c>
       <c r="AB3" t="n">
-        <v>62975</v>
+        <v>78615</v>
       </c>
       <c r="AC3" t="n">
         <v>0.01</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.92</v>
+        <v>0.76</v>
       </c>
       <c r="AE3" t="n">
-        <v>9720</v>
+        <v>12456</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45774</v>
+      <c r="A4" s="2" t="n">
+        <v>45865</v>
       </c>
       <c r="B4" t="n">
-        <v>141.76</v>
+        <v>164</v>
       </c>
       <c r="C4" t="n">
-        <v>13.15</v>
+        <v>53.57</v>
       </c>
       <c r="D4" t="n">
-        <v>7.6</v>
+        <v>1.87</v>
       </c>
       <c r="E4" t="n">
-        <v>22249</v>
+        <v>29109</v>
       </c>
       <c r="F4" t="n">
-        <v>42.61</v>
+        <v>56.53</v>
       </c>
       <c r="G4" t="n">
-        <v>31.75</v>
+        <v>43.27</v>
       </c>
       <c r="H4" t="n">
-        <v>2661624900</v>
+        <v>4333249440</v>
       </c>
       <c r="I4" t="n">
-        <v>10285</v>
+        <v>10598</v>
       </c>
       <c r="J4" t="n">
-        <v>53691</v>
+        <v>56791</v>
       </c>
       <c r="K4" t="n">
-        <v>-43406</v>
+        <v>-46193</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.54</v>
+        <v>-0.5</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.52</v>
+        <v>-0.46</v>
       </c>
       <c r="N4" t="n">
-        <v>33.4</v>
+        <v>47.2</v>
       </c>
       <c r="O4" t="n">
-        <v>82.97</v>
+        <v>81</v>
       </c>
       <c r="P4" t="n">
-        <v>72.14</v>
+        <v>69.58</v>
       </c>
       <c r="Q4" t="n">
-        <v>27414</v>
+        <v>15365</v>
       </c>
       <c r="R4" t="n">
-        <v>-5216</v>
+        <v>-7127</v>
       </c>
       <c r="S4" t="n">
-        <v>-15553</v>
+        <v>-11833</v>
       </c>
       <c r="T4" t="n">
-        <v>26187</v>
+        <v>13470</v>
       </c>
       <c r="U4" t="n">
-        <v>1227</v>
+        <v>1895</v>
       </c>
       <c r="V4" t="n">
-        <v>1454</v>
+        <v>2721</v>
       </c>
       <c r="W4" t="n">
-        <v>3989</v>
+        <v>4291</v>
       </c>
       <c r="X4" t="n">
-        <v>14643</v>
+        <v>17481</v>
       </c>
       <c r="Y4" t="n">
-        <v>63393</v>
+        <v>77962</v>
       </c>
       <c r="Z4" t="n">
-        <v>12.03</v>
+        <v>36.97</v>
       </c>
       <c r="AA4" t="n">
-        <v>73337</v>
+        <v>66129</v>
       </c>
       <c r="AB4" t="n">
-        <v>72769</v>
+        <v>62975</v>
       </c>
       <c r="AC4" t="n">
         <v>0.01</v>
       </c>
       <c r="AD4" t="n">
-        <v>1.3</v>
+        <v>0.92</v>
       </c>
       <c r="AE4" t="n">
-        <v>14095</v>
+        <v>9720</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45592</v>
+      <c r="A5" s="2" t="n">
+        <v>45774</v>
       </c>
       <c r="B5" t="n">
-        <v>168.61</v>
+        <v>141.75</v>
       </c>
       <c r="C5" t="n">
-        <v>11.79</v>
+        <v>13.15</v>
       </c>
       <c r="D5" t="n">
-        <v>8.48</v>
+        <v>7.6</v>
       </c>
       <c r="E5" t="n">
-        <v>22347</v>
+        <v>22249</v>
       </c>
       <c r="F5" t="n">
-        <v>55.04</v>
+        <v>42.61</v>
       </c>
       <c r="G5" t="n">
-        <v>49.33</v>
+        <v>31.75</v>
       </c>
       <c r="H5" t="n">
-        <v>3255774430</v>
+        <v>2661380490</v>
       </c>
       <c r="I5" t="n">
-        <v>10225</v>
+        <v>10285</v>
       </c>
       <c r="J5" t="n">
-        <v>38487</v>
+        <v>53691</v>
       </c>
       <c r="K5" t="n">
-        <v>-28262</v>
+        <v>-43406</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.41</v>
+        <v>-0.54</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.43</v>
+        <v>-0.52</v>
       </c>
       <c r="N5" t="n">
-        <v>47.23</v>
+        <v>33.4</v>
       </c>
       <c r="O5" t="n">
-        <v>91.09999999999999</v>
+        <v>82.97</v>
       </c>
       <c r="P5" t="n">
-        <v>76.90000000000001</v>
+        <v>72.14</v>
       </c>
       <c r="Q5" t="n">
-        <v>17627</v>
+        <v>27414</v>
       </c>
       <c r="R5" t="n">
-        <v>-4346</v>
+        <v>-5216</v>
       </c>
       <c r="S5" t="n">
-        <v>-12745</v>
+        <v>-15553</v>
       </c>
       <c r="T5" t="n">
-        <v>16814</v>
+        <v>26187</v>
       </c>
       <c r="U5" t="n">
-        <v>813</v>
+        <v>1227</v>
       </c>
       <c r="V5" t="n">
-        <v>744</v>
+        <v>1454</v>
       </c>
       <c r="W5" t="n">
-        <v>3390</v>
+        <v>3989</v>
       </c>
       <c r="X5" t="n">
-        <v>12238</v>
+        <v>14643</v>
       </c>
       <c r="Y5" t="n">
-        <v>51161</v>
+        <v>63393</v>
       </c>
       <c r="Z5" t="n">
-        <v>26.54</v>
+        <v>12.03</v>
       </c>
       <c r="AA5" t="n">
-        <v>54741</v>
+        <v>73337</v>
       </c>
       <c r="AB5" t="n">
-        <v>54655</v>
+        <v>72769</v>
       </c>
       <c r="AC5" t="n">
         <v>0.01</v>
       </c>
       <c r="AD5" t="n">
-        <v>1.27</v>
+        <v>1.3</v>
       </c>
       <c r="AE5" t="n">
-        <v>10997</v>
+        <v>14095</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>45501</v>
+      <c r="A6" s="2" t="n">
+        <v>45592</v>
       </c>
       <c r="B6" t="n">
-        <v>173.2</v>
+        <v>168.61</v>
       </c>
       <c r="C6" t="n">
-        <v>9.02</v>
+        <v>11.79</v>
       </c>
       <c r="D6" t="n">
-        <v>11.09</v>
+        <v>8.48</v>
       </c>
       <c r="E6" t="n">
-        <v>19075</v>
+        <v>22347</v>
       </c>
       <c r="F6" t="n">
-        <v>55.26</v>
+        <v>55.04</v>
       </c>
       <c r="G6" t="n">
-        <v>49.35</v>
+        <v>49.33</v>
       </c>
       <c r="H6" t="n">
-        <v>2874888660</v>
+        <v>3255774430</v>
       </c>
       <c r="I6" t="n">
-        <v>10015</v>
+        <v>10225</v>
       </c>
       <c r="J6" t="n">
-        <v>34800</v>
+        <v>38487</v>
       </c>
       <c r="K6" t="n">
-        <v>-24785</v>
+        <v>-28262</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.46</v>
+        <v>-0.41</v>
       </c>
       <c r="M6" t="n">
         <v>-0.43</v>
       </c>
       <c r="N6" t="n">
-        <v>53.35</v>
+        <v>47.23</v>
       </c>
       <c r="O6" t="n">
-        <v>80.66</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="P6" t="n">
-        <v>67.01000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="Q6" t="n">
-        <v>14488</v>
+        <v>17627</v>
       </c>
       <c r="R6" t="n">
-        <v>-3184</v>
+        <v>-4346</v>
       </c>
       <c r="S6" t="n">
-        <v>-10320</v>
+        <v>-12745</v>
       </c>
       <c r="T6" t="n">
-        <v>13511</v>
+        <v>16814</v>
       </c>
       <c r="U6" t="n">
-        <v>977</v>
+        <v>813</v>
       </c>
       <c r="V6" t="n">
-        <v>333</v>
+        <v>744</v>
       </c>
       <c r="W6" t="n">
-        <v>3090</v>
+        <v>3390</v>
       </c>
       <c r="X6" t="n">
-        <v>10477</v>
+        <v>12238</v>
       </c>
       <c r="Y6" t="n">
-        <v>45664</v>
+        <v>51161</v>
       </c>
       <c r="Z6" t="n">
-        <v>30.29</v>
+        <v>26.54</v>
       </c>
       <c r="AA6" t="n">
-        <v>40719</v>
+        <v>54741</v>
       </c>
       <c r="AB6" t="n">
-        <v>41894</v>
+        <v>54655</v>
       </c>
       <c r="AC6" t="n">
         <v>0.01</v>
       </c>
       <c r="AD6" t="n">
-        <v>1.48</v>
+        <v>1.27</v>
       </c>
       <c r="AE6" t="n">
-        <v>7158</v>
+        <v>10997</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45410</v>
+      <c r="A7" s="2" t="n">
+        <v>45501</v>
       </c>
       <c r="B7" t="n">
-        <v>142.88</v>
+        <v>173.18</v>
       </c>
       <c r="C7" t="n">
-        <v>65.81999999999999</v>
+        <v>9.02</v>
       </c>
       <c r="D7" t="n">
-        <v>1.52</v>
+        <v>11.09</v>
       </c>
       <c r="E7" t="n">
-        <v>17319</v>
+        <v>19075</v>
       </c>
       <c r="F7" t="n">
-        <v>57.14</v>
+        <v>55.26</v>
       </c>
       <c r="G7" t="n">
-        <v>43.27</v>
+        <v>49.35</v>
       </c>
       <c r="H7" t="n">
-        <v>2126183200</v>
+        <v>2874642880</v>
       </c>
       <c r="I7" t="n">
-        <v>11237</v>
+        <v>10015</v>
       </c>
       <c r="J7" t="n">
-        <v>31438</v>
+        <v>34800</v>
       </c>
       <c r="K7" t="n">
-        <v>-20201</v>
+        <v>-24785</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.53</v>
+        <v>-0.46</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.41</v>
+        <v>-0.43</v>
       </c>
       <c r="N7" t="n">
-        <v>56.79</v>
+        <v>53.35</v>
       </c>
       <c r="O7" t="n">
-        <v>65.84</v>
+        <v>80.66</v>
       </c>
       <c r="P7" t="n">
-        <v>52.39</v>
+        <v>67.01000000000001</v>
       </c>
       <c r="Q7" t="n">
-        <v>15345</v>
+        <v>14488</v>
       </c>
       <c r="R7" t="n">
-        <v>-5693</v>
+        <v>-3184</v>
       </c>
       <c r="S7" t="n">
-        <v>-9345</v>
+        <v>-10320</v>
       </c>
       <c r="T7" t="n">
-        <v>14976</v>
+        <v>13511</v>
       </c>
       <c r="U7" t="n">
-        <v>369</v>
+        <v>977</v>
       </c>
       <c r="V7" t="n">
-        <v>-347</v>
+        <v>333</v>
       </c>
       <c r="W7" t="n">
-        <v>2720</v>
+        <v>3090</v>
       </c>
       <c r="X7" t="n">
-        <v>8582</v>
+        <v>10477</v>
       </c>
       <c r="Y7" t="n">
-        <v>38506</v>
+        <v>45664</v>
       </c>
       <c r="Z7" t="n">
-        <v>29.48</v>
+        <v>30.29</v>
       </c>
       <c r="AA7" t="n">
-        <v>30709</v>
+        <v>40719</v>
       </c>
       <c r="AB7" t="n">
-        <v>30837</v>
+        <v>41894</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.66</v>
+        <v>1.48</v>
       </c>
       <c r="AE7" t="n">
-        <v>7740</v>
+        <v>7158</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45228</v>
+      <c r="A8" s="2" t="n">
+        <v>45410</v>
       </c>
       <c r="B8" t="n">
-        <v>108.81</v>
+        <v>142.86</v>
       </c>
       <c r="C8" t="n">
-        <v>55.44</v>
+        <v>65.81999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>1.8</v>
+        <v>1.52</v>
       </c>
       <c r="E8" t="n">
-        <v>10789</v>
+        <v>17319</v>
       </c>
       <c r="F8" t="n">
-        <v>51.01</v>
+        <v>57.14</v>
       </c>
       <c r="G8" t="n">
-        <v>30.23</v>
+        <v>43.26</v>
       </c>
       <c r="H8" t="n">
-        <v>1005710000</v>
+        <v>2125937000</v>
       </c>
       <c r="I8" t="n">
-        <v>11027</v>
+        <v>11237</v>
       </c>
       <c r="J8" t="n">
-        <v>18281</v>
+        <v>31438</v>
       </c>
       <c r="K8" t="n">
-        <v>-7254</v>
+        <v>-20201</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.34</v>
+        <v>-0.53</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.22</v>
+        <v>-0.41</v>
       </c>
       <c r="N8" t="n">
-        <v>47.15</v>
+        <v>56.78</v>
       </c>
       <c r="O8" t="n">
-        <v>54.57</v>
+        <v>65.84</v>
       </c>
       <c r="P8" t="n">
-        <v>40.16</v>
+        <v>52.39</v>
       </c>
       <c r="Q8" t="n">
-        <v>7332</v>
+        <v>15345</v>
       </c>
       <c r="R8" t="n">
-        <v>-3170</v>
+        <v>-5693</v>
       </c>
       <c r="S8" t="n">
-        <v>-4525</v>
+        <v>-9345</v>
       </c>
       <c r="T8" t="n">
-        <v>7054</v>
+        <v>14976</v>
       </c>
       <c r="U8" t="n">
-        <v>278</v>
+        <v>369</v>
       </c>
       <c r="V8" t="n">
-        <v>-182</v>
+        <v>-347</v>
       </c>
       <c r="W8" t="n">
-        <v>2294</v>
+        <v>2720</v>
       </c>
       <c r="X8" t="n">
-        <v>7972</v>
+        <v>8582</v>
       </c>
       <c r="Y8" t="n">
-        <v>23557</v>
+        <v>38506</v>
       </c>
       <c r="Z8" t="n">
-        <v>63.16</v>
+        <v>29.48</v>
       </c>
       <c r="AA8" t="n">
-        <v>13823</v>
+        <v>30709</v>
       </c>
       <c r="AB8" t="n">
-        <v>14451</v>
+        <v>30837</v>
       </c>
       <c r="AC8" t="n">
         <v>0.04</v>
       </c>
       <c r="AD8" t="n">
-        <v>1.05</v>
+        <v>0.66</v>
       </c>
       <c r="AE8" t="n">
-        <v>3807</v>
+        <v>7740</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45137</v>
+      <c r="A9" s="2" t="n">
+        <v>45228</v>
       </c>
       <c r="B9" t="n">
-        <v>186.63</v>
+        <v>108.81</v>
       </c>
       <c r="C9" t="n">
-        <v>120.98</v>
+        <v>55.44</v>
       </c>
       <c r="D9" t="n">
-        <v>0.83</v>
+        <v>1.8</v>
       </c>
       <c r="E9" t="n">
-        <v>7165</v>
+        <v>10789</v>
       </c>
       <c r="F9" t="n">
-        <v>45.81</v>
+        <v>51.01</v>
       </c>
       <c r="G9" t="n">
-        <v>42</v>
+        <v>30.23</v>
       </c>
       <c r="H9" t="n">
-        <v>1154891000</v>
+        <v>1005710000</v>
       </c>
       <c r="I9" t="n">
-        <v>10954</v>
+        <v>11027</v>
       </c>
       <c r="J9" t="n">
-        <v>16023</v>
+        <v>18281</v>
       </c>
       <c r="K9" t="n">
-        <v>-5069</v>
+        <v>-7254</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.44</v>
+        <v>-0.34</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.18</v>
+        <v>-0.22</v>
       </c>
       <c r="N9" t="n">
-        <v>100.23</v>
+        <v>47.15</v>
       </c>
       <c r="O9" t="n">
-        <v>34.79</v>
+        <v>54.57</v>
       </c>
       <c r="P9" t="n">
-        <v>24.26</v>
+        <v>40.16</v>
       </c>
       <c r="Q9" t="n">
-        <v>6348</v>
+        <v>7332</v>
       </c>
       <c r="R9" t="n">
-        <v>-446</v>
+        <v>-3170</v>
       </c>
       <c r="S9" t="n">
-        <v>-5099</v>
+        <v>-4525</v>
       </c>
       <c r="T9" t="n">
-        <v>6059</v>
+        <v>7054</v>
       </c>
       <c r="U9" t="n">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="V9" t="n">
-        <v>-33</v>
+        <v>-182</v>
       </c>
       <c r="W9" t="n">
-        <v>2040</v>
+        <v>2294</v>
       </c>
       <c r="X9" t="n">
-        <v>7651</v>
+        <v>7972</v>
       </c>
       <c r="Y9" t="n">
-        <v>18463</v>
+        <v>23557</v>
       </c>
       <c r="Z9" t="n">
-        <v>91.86999999999999</v>
+        <v>63.16</v>
       </c>
       <c r="AA9" t="n">
-        <v>7430</v>
+        <v>13823</v>
       </c>
       <c r="AB9" t="n">
-        <v>8013</v>
+        <v>14451</v>
       </c>
       <c r="AC9" t="n">
         <v>0.04</v>
       </c>
       <c r="AD9" t="n">
-        <v>1.62</v>
+        <v>1.05</v>
       </c>
       <c r="AE9" t="n">
-        <v>3067</v>
+        <v>3807</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>45046</v>
+      <c r="A10" s="2" t="n">
+        <v>45137</v>
       </c>
       <c r="B10" t="n">
-        <v>335.26</v>
+        <v>186.59</v>
       </c>
       <c r="C10" t="n">
-        <v>137.96</v>
+        <v>120.96</v>
       </c>
       <c r="D10" t="n">
-        <v>0.72</v>
+        <v>0.83</v>
       </c>
       <c r="E10" t="n">
-        <v>2524</v>
+        <v>7165</v>
       </c>
       <c r="F10" t="n">
-        <v>28.41</v>
+        <v>45.81</v>
       </c>
       <c r="G10" t="n">
-        <v>27.93</v>
+        <v>41.99</v>
       </c>
       <c r="H10" t="n">
-        <v>684931000</v>
+        <v>1154643700</v>
       </c>
       <c r="I10" t="n">
-        <v>12080</v>
+        <v>10954</v>
       </c>
       <c r="J10" t="n">
-        <v>15320</v>
+        <v>16023</v>
       </c>
       <c r="K10" t="n">
-        <v>-3240</v>
+        <v>-5069</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.49</v>
+        <v>-0.44</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.13</v>
+        <v>-0.18</v>
       </c>
       <c r="N10" t="n">
-        <v>104.11</v>
+        <v>100.21</v>
       </c>
       <c r="O10" t="n">
-        <v>20.38</v>
+        <v>34.79</v>
       </c>
       <c r="P10" t="n">
-        <v>13.67</v>
+        <v>24.26</v>
       </c>
       <c r="Q10" t="n">
-        <v>2911</v>
+        <v>6348</v>
       </c>
       <c r="R10" t="n">
-        <v>-841</v>
+        <v>-446</v>
       </c>
       <c r="S10" t="n">
-        <v>-380</v>
+        <v>-5099</v>
       </c>
       <c r="T10" t="n">
-        <v>2663</v>
+        <v>6059</v>
       </c>
       <c r="U10" t="n">
-        <v>248</v>
+        <v>289</v>
       </c>
       <c r="V10" t="n">
-        <v>70</v>
+        <v>-33</v>
       </c>
       <c r="W10" t="n">
-        <v>1875</v>
+        <v>2040</v>
       </c>
       <c r="X10" t="n">
-        <v>7332</v>
+        <v>7651</v>
       </c>
       <c r="Y10" t="n">
-        <v>17623</v>
+        <v>18463</v>
       </c>
       <c r="Z10" t="n">
-        <v>151.17</v>
+        <v>91.86999999999999</v>
       </c>
       <c r="AA10" t="n">
-        <v>4696</v>
+        <v>7430</v>
       </c>
       <c r="AB10" t="n">
-        <v>4423</v>
+        <v>8013</v>
       </c>
       <c r="AC10" t="n">
         <v>0.04</v>
       </c>
       <c r="AD10" t="n">
-        <v>4.85</v>
+        <v>1.62</v>
       </c>
       <c r="AE10" t="n">
-        <v>0</v>
+        <v>3067</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>44864</v>
+      <c r="A11" s="2" t="n">
+        <v>45046</v>
       </c>
       <c r="B11" t="n">
-        <v>492.22</v>
+        <v>335.14</v>
       </c>
       <c r="C11" t="n">
-        <v>62.12</v>
+        <v>137.91</v>
       </c>
       <c r="D11" t="n">
-        <v>1.61</v>
+        <v>0.73</v>
       </c>
       <c r="E11" t="n">
-        <v>1007</v>
+        <v>2524</v>
       </c>
       <c r="F11" t="n">
-        <v>11.47</v>
+        <v>28.41</v>
       </c>
       <c r="G11" t="n">
-        <v>15.67</v>
+        <v>27.92</v>
       </c>
       <c r="H11" t="n">
-        <v>334708400</v>
+        <v>684684000</v>
       </c>
       <c r="I11" t="n">
-        <v>11904</v>
+        <v>12080</v>
       </c>
       <c r="J11" t="n">
-        <v>13143</v>
+        <v>15320</v>
       </c>
       <c r="K11" t="n">
-        <v>-1239</v>
+        <v>-3240</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.18</v>
+        <v>-0.49</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.06</v>
+        <v>-0.13</v>
       </c>
       <c r="N11" t="n">
-        <v>47.62</v>
+        <v>104.07</v>
       </c>
       <c r="O11" t="n">
-        <v>25.38</v>
+        <v>20.38</v>
       </c>
       <c r="P11" t="n">
-        <v>16.62</v>
+        <v>13.67</v>
       </c>
       <c r="Q11" t="n">
-        <v>392</v>
+        <v>2911</v>
       </c>
       <c r="R11" t="n">
-        <v>3148</v>
+        <v>-841</v>
       </c>
       <c r="S11" t="n">
-        <v>-3753</v>
+        <v>-380</v>
       </c>
       <c r="T11" t="n">
-        <v>-138</v>
+        <v>2663</v>
       </c>
       <c r="U11" t="n">
-        <v>530</v>
+        <v>248</v>
       </c>
       <c r="V11" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="W11" t="n">
-        <v>1945</v>
+        <v>1875</v>
       </c>
       <c r="X11" t="n">
-        <v>6920</v>
+        <v>7332</v>
       </c>
       <c r="Y11" t="n">
-        <v>16368</v>
+        <v>17623</v>
       </c>
       <c r="Z11" t="n">
-        <v>150.65</v>
+        <v>151.17</v>
       </c>
       <c r="AA11" t="n">
-        <v>2875</v>
+        <v>4696</v>
       </c>
       <c r="AB11" t="n">
-        <v>4104</v>
+        <v>4423</v>
       </c>
       <c r="AC11" t="n">
         <v>0.04</v>
       </c>
       <c r="AD11" t="n">
-        <v>14.71</v>
+        <v>4.85</v>
       </c>
       <c r="AE11" t="n">
-        <v>3485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>44773</v>
+      <c r="A12" s="2" t="n">
+        <v>44864</v>
       </c>
       <c r="B12" t="n">
-        <v>689.55</v>
+        <v>492.22</v>
       </c>
       <c r="C12" t="n">
-        <v>63.61</v>
+        <v>62.12</v>
       </c>
       <c r="D12" t="n">
-        <v>1.57</v>
+        <v>1.61</v>
       </c>
       <c r="E12" t="n">
-        <v>877</v>
+        <v>1007</v>
       </c>
       <c r="F12" t="n">
-        <v>9.789999999999999</v>
+        <v>11.47</v>
       </c>
       <c r="G12" t="n">
-        <v>18.96</v>
+        <v>15.67</v>
       </c>
       <c r="H12" t="n">
-        <v>452343499.9999999</v>
+        <v>334708400</v>
       </c>
       <c r="I12" t="n">
-        <v>11837</v>
+        <v>11904</v>
       </c>
       <c r="J12" t="n">
-        <v>17037</v>
+        <v>13143</v>
       </c>
       <c r="K12" t="n">
-        <v>-5200</v>
+        <v>-1239</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.59</v>
+        <v>-0.18</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.22</v>
+        <v>-0.06</v>
       </c>
       <c r="N12" t="n">
-        <v>52.12</v>
+        <v>47.62</v>
       </c>
       <c r="O12" t="n">
-        <v>29.82</v>
+        <v>25.38</v>
       </c>
       <c r="P12" t="n">
-        <v>20.4</v>
+        <v>16.62</v>
       </c>
       <c r="Q12" t="n">
-        <v>1270</v>
+        <v>392</v>
       </c>
       <c r="R12" t="n">
-        <v>1618</v>
+        <v>3148</v>
       </c>
       <c r="S12" t="n">
-        <v>-3762</v>
+        <v>-3753</v>
       </c>
       <c r="T12" t="n">
-        <v>837</v>
+        <v>-138</v>
       </c>
       <c r="U12" t="n">
-        <v>433</v>
+        <v>530</v>
       </c>
       <c r="V12" t="n">
-        <v>-97</v>
+        <v>130</v>
       </c>
       <c r="W12" t="n">
-        <v>1824</v>
+        <v>1945</v>
       </c>
       <c r="X12" t="n">
-        <v>5993</v>
+        <v>6920</v>
       </c>
       <c r="Y12" t="n">
-        <v>19845</v>
+        <v>16368</v>
       </c>
       <c r="Z12" t="n">
-        <v>87.98</v>
+        <v>150.65</v>
       </c>
       <c r="AA12" t="n">
-        <v>10772</v>
+        <v>2875</v>
       </c>
       <c r="AB12" t="n">
-        <v>7165</v>
+        <v>4104</v>
       </c>
       <c r="AC12" t="n">
         <v>0.04</v>
       </c>
       <c r="AD12" t="n">
-        <v>15.24</v>
+        <v>14.71</v>
       </c>
       <c r="AE12" t="n">
-        <v>3345</v>
+        <v>3485</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>44652</v>
+      <c r="A13" s="2" t="n">
+        <v>44773</v>
       </c>
       <c r="B13" t="n">
-        <v>286.69</v>
+        <v>689.55</v>
       </c>
       <c r="C13" t="n">
-        <v>32.65</v>
+        <v>63.61</v>
       </c>
       <c r="D13" t="n">
-        <v>3.06</v>
+        <v>1.57</v>
       </c>
       <c r="E13" t="n">
-        <v>2202</v>
+        <v>877</v>
       </c>
       <c r="F13" t="n">
-        <v>19.52</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>17.63</v>
+        <v>18.96</v>
       </c>
       <c r="H13" t="n">
-        <v>463860600.0000001</v>
+        <v>452343499.9999999</v>
       </c>
       <c r="I13" t="n">
-        <v>11846</v>
+        <v>11837</v>
       </c>
       <c r="J13" t="n">
-        <v>20338</v>
+        <v>17037</v>
       </c>
       <c r="K13" t="n">
-        <v>-8492</v>
+        <v>-5200</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.84</v>
+        <v>-0.59</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.32</v>
+        <v>-0.22</v>
       </c>
       <c r="N13" t="n">
-        <v>46.59</v>
+        <v>52.12</v>
       </c>
       <c r="O13" t="n">
-        <v>31.79</v>
+        <v>29.82</v>
       </c>
       <c r="P13" t="n">
-        <v>22.08</v>
+        <v>20.4</v>
       </c>
       <c r="Q13" t="n">
-        <v>1731</v>
+        <v>1270</v>
       </c>
       <c r="R13" t="n">
-        <v>2612</v>
+        <v>1618</v>
       </c>
       <c r="S13" t="n">
-        <v>-2446</v>
+        <v>-3762</v>
       </c>
       <c r="T13" t="n">
-        <v>1370</v>
+        <v>837</v>
       </c>
       <c r="U13" t="n">
-        <v>361</v>
+        <v>433</v>
       </c>
       <c r="V13" t="n">
-        <v>-135</v>
+        <v>-97</v>
       </c>
       <c r="W13" t="n">
-        <v>1618</v>
+        <v>1824</v>
       </c>
       <c r="X13" t="n">
-        <v>5284</v>
+        <v>5993</v>
       </c>
       <c r="Y13" t="n">
-        <v>24013</v>
+        <v>19845</v>
       </c>
       <c r="Z13" t="n">
-        <v>88.73</v>
+        <v>87.98</v>
       </c>
       <c r="AA13" t="n">
-        <v>10288</v>
+        <v>10772</v>
       </c>
       <c r="AB13" t="n">
-        <v>5956</v>
+        <v>7165</v>
       </c>
       <c r="AC13" t="n">
         <v>0.04</v>
       </c>
       <c r="AD13" t="n">
-        <v>6.18</v>
+        <v>15.24</v>
       </c>
       <c r="AE13" t="n">
-        <v>1996</v>
+        <v>3345</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>44500</v>
+      <c r="A14" s="2" t="n">
+        <v>44652</v>
       </c>
       <c r="B14" t="n">
-        <v>258.72</v>
+        <v>286.69</v>
       </c>
       <c r="C14" t="n">
-        <v>35.53</v>
+        <v>32.65</v>
       </c>
       <c r="D14" t="n">
-        <v>2.81</v>
+        <v>3.06</v>
       </c>
       <c r="E14" t="n">
-        <v>2969</v>
+        <v>2202</v>
       </c>
       <c r="F14" t="n">
-        <v>34.69</v>
+        <v>19.52</v>
       </c>
       <c r="G14" t="n">
-        <v>26.8</v>
+        <v>17.63</v>
       </c>
       <c r="H14" t="n">
-        <v>637494900</v>
+        <v>463860600.0000001</v>
       </c>
       <c r="I14" t="n">
-        <v>11827</v>
+        <v>11846</v>
       </c>
       <c r="J14" t="n">
-        <v>19298</v>
+        <v>20338</v>
       </c>
       <c r="K14" t="n">
-        <v>-7471</v>
+        <v>-8492</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.78</v>
+        <v>-0.84</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.31</v>
+        <v>-0.32</v>
       </c>
       <c r="N14" t="n">
-        <v>66.95</v>
+        <v>46.59</v>
       </c>
       <c r="O14" t="n">
-        <v>33.98</v>
+        <v>31.79</v>
       </c>
       <c r="P14" t="n">
-        <v>22.82</v>
+        <v>22.08</v>
       </c>
       <c r="Q14" t="n">
-        <v>1519</v>
+        <v>1731</v>
       </c>
       <c r="R14" t="n">
-        <v>-4439</v>
+        <v>2612</v>
       </c>
       <c r="S14" t="n">
-        <v>-1420</v>
+        <v>-2446</v>
       </c>
       <c r="T14" t="n">
-        <v>1297</v>
+        <v>1370</v>
       </c>
       <c r="U14" t="n">
-        <v>222</v>
+        <v>361</v>
       </c>
       <c r="V14" t="n">
-        <v>384</v>
+        <v>-135</v>
       </c>
       <c r="W14" t="n">
-        <v>1403</v>
+        <v>1618</v>
       </c>
       <c r="X14" t="n">
-        <v>5232</v>
+        <v>5284</v>
       </c>
       <c r="Y14" t="n">
-        <v>22194</v>
+        <v>24013</v>
       </c>
       <c r="Z14" t="n">
-        <v>86.39</v>
+        <v>88.73</v>
       </c>
       <c r="AA14" t="n">
-        <v>9887</v>
+        <v>10288</v>
       </c>
       <c r="AB14" t="n">
-        <v>5734</v>
+        <v>5956</v>
       </c>
       <c r="AC14" t="n">
         <v>0.04</v>
       </c>
       <c r="AD14" t="n">
-        <v>4.06</v>
+        <v>6.18</v>
       </c>
       <c r="AE14" t="n">
-        <v>0</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>44378</v>
+      <c r="A15" s="2" t="n">
+        <v>44500</v>
       </c>
       <c r="B15" t="n">
-        <v>204.35</v>
+        <v>258.72</v>
       </c>
       <c r="C15" t="n">
-        <v>27.03</v>
+        <v>35.53</v>
       </c>
       <c r="D15" t="n">
-        <v>3.7</v>
+        <v>2.81</v>
       </c>
       <c r="E15" t="n">
-        <v>2730</v>
+        <v>2969</v>
       </c>
       <c r="F15" t="n">
-        <v>36.48</v>
+        <v>34.69</v>
       </c>
       <c r="G15" t="n">
-        <v>22.95</v>
+        <v>26.8</v>
       </c>
       <c r="H15" t="n">
-        <v>485137800.0000001</v>
+        <v>637494900</v>
       </c>
       <c r="I15" t="n">
-        <v>12791</v>
+        <v>11827</v>
       </c>
       <c r="J15" t="n">
-        <v>19654</v>
+        <v>19298</v>
       </c>
       <c r="K15" t="n">
-        <v>-6863</v>
+        <v>-7471</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.89</v>
+        <v>-0.78</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.32</v>
+        <v>-0.31</v>
       </c>
       <c r="N15" t="n">
-        <v>63.74</v>
+        <v>66.95</v>
       </c>
       <c r="O15" t="n">
-        <v>29.53</v>
+        <v>33.98</v>
       </c>
       <c r="P15" t="n">
-        <v>18.56</v>
+        <v>22.82</v>
       </c>
       <c r="Q15" t="n">
-        <v>2682</v>
+        <v>1519</v>
       </c>
       <c r="R15" t="n">
-        <v>-2533</v>
+        <v>-4439</v>
       </c>
       <c r="S15" t="n">
-        <v>4501</v>
+        <v>-1420</v>
       </c>
       <c r="T15" t="n">
-        <v>2499</v>
+        <v>1297</v>
       </c>
       <c r="U15" t="n">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="V15" t="n">
-        <v>56</v>
+        <v>384</v>
       </c>
       <c r="W15" t="n">
-        <v>1245</v>
+        <v>1403</v>
       </c>
       <c r="X15" t="n">
-        <v>4498</v>
+        <v>5232</v>
       </c>
       <c r="Y15" t="n">
-        <v>21358</v>
+        <v>22194</v>
       </c>
       <c r="Z15" t="n">
-        <v>78.73999999999999</v>
+        <v>86.39</v>
       </c>
       <c r="AA15" t="n">
-        <v>10704</v>
+        <v>9887</v>
       </c>
       <c r="AB15" t="n">
-        <v>5878</v>
+        <v>5734</v>
       </c>
       <c r="AC15" t="n">
         <v>0.04</v>
       </c>
       <c r="AD15" t="n">
-        <v>4.17</v>
+        <v>4.06</v>
       </c>
       <c r="AE15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
+        <v>44378</v>
+      </c>
+      <c r="B16" t="n">
+        <v>204.25</v>
+      </c>
+      <c r="C16" t="n">
+        <v>27.01</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2730</v>
+      </c>
+      <c r="F16" t="n">
+        <v>36.48</v>
+      </c>
+      <c r="G16" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="H16" t="n">
+        <v>484888500</v>
+      </c>
+      <c r="I16" t="n">
+        <v>12791</v>
+      </c>
+      <c r="J16" t="n">
+        <v>19654</v>
+      </c>
+      <c r="K16" t="n">
+        <v>-6863</v>
+      </c>
+      <c r="L16" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="N16" t="n">
+        <v>63.71</v>
+      </c>
+      <c r="O16" t="n">
+        <v>29.53</v>
+      </c>
+      <c r="P16" t="n">
+        <v>18.56</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>2682</v>
+      </c>
+      <c r="R16" t="n">
+        <v>-2533</v>
+      </c>
+      <c r="S16" t="n">
+        <v>4501</v>
+      </c>
+      <c r="T16" t="n">
+        <v>2499</v>
+      </c>
+      <c r="U16" t="n">
+        <v>183</v>
+      </c>
+      <c r="V16" t="n">
+        <v>56</v>
+      </c>
+      <c r="W16" t="n">
+        <v>1245</v>
+      </c>
+      <c r="X16" t="n">
+        <v>4498</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>21358</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>78.73999999999999</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>10704</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>5878</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>44288</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>194.48</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C17" t="n">
         <v>77.36</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>1.29</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E17" t="n">
         <v>2237</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F17" t="n">
         <v>33.77</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G17" t="n">
         <v>19.81</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H17" t="n">
         <v>371854800.0000001</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I17" t="n">
         <v>7738</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J17" t="n">
         <v>12667</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K17" t="n">
         <v>-4929</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L17" t="n">
         <v>-0.8100000000000001</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M17" t="n">
         <v>-0.26</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N17" t="n">
         <v>62.05</v>
       </c>
-      <c r="O16" t="n">
+      <c r="O17" t="n">
         <v>25.5</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P17" t="n">
         <v>18.05</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q17" t="n">
         <v>1874</v>
       </c>
-      <c r="R16" t="n">
+      <c r="R17" t="n">
         <v>-1272</v>
       </c>
-      <c r="S16" t="n">
+      <c r="S17" t="n">
         <v>-471</v>
       </c>
-      <c r="T16" t="n">
+      <c r="T17" t="n">
         <v>1576</v>
       </c>
-      <c r="U16" t="n">
+      <c r="U17" t="n">
         <v>298</v>
       </c>
-      <c r="V16" t="n">
+      <c r="V17" t="n">
         <v>52</v>
       </c>
-      <c r="W16" t="n">
+      <c r="W17" t="n">
         <v>1153</v>
       </c>
-      <c r="X16" t="n">
+      <c r="X17" t="n">
         <v>3984</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="Y17" t="n">
         <v>14123</v>
       </c>
-      <c r="Z16" t="n">
+      <c r="Z17" t="n">
         <v>96.03</v>
       </c>
-      <c r="AA16" t="n">
+      <c r="AA17" t="n">
         <v>9094</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AB17" t="n">
         <v>3995</v>
       </c>
-      <c r="AC16" t="n">
+      <c r="AC17" t="n">
         <v>0.16</v>
       </c>
-      <c r="AD16" t="n">
+      <c r="AD17" t="n">
         <v>5.18</v>
       </c>
-      <c r="AE16" t="n">
+      <c r="AE17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualizei os dados do 2Q27 da NVDA
</commit_message>
<xml_diff>
--- a/analise_eua/semicondutores/nvidia/nvda_indicators.xlsx
+++ b/analise_eua/semicondutores/nvidia/nvda_indicators.xlsx
@@ -592,10 +592,10 @@
         <v>2026</v>
       </c>
       <c r="B2" t="n">
-        <v>38.77</v>
+        <v>38.73</v>
       </c>
       <c r="C2" t="n">
-        <v>38.77</v>
+        <v>38.72</v>
       </c>
       <c r="D2" t="n">
         <v>2.58</v>
@@ -607,10 +607,10 @@
         <v>55.6</v>
       </c>
       <c r="G2" t="n">
-        <v>29.59</v>
+        <v>29.55</v>
       </c>
       <c r="H2" t="n">
-        <v>4655492080</v>
+        <v>4650133100.000001</v>
       </c>
       <c r="I2" t="n">
         <v>11412</v>
@@ -628,7 +628,7 @@
         <v>-0.33</v>
       </c>
       <c r="N2" t="n">
-        <v>35.33</v>
+        <v>35.29</v>
       </c>
       <c r="O2" t="n">
         <v>76.33</v>
@@ -687,13 +687,13 @@
         <v>2025</v>
       </c>
       <c r="B3" t="n">
-        <v>40.44</v>
+        <v>40.39</v>
       </c>
       <c r="C3" t="n">
-        <v>40.41</v>
+        <v>40.37</v>
       </c>
       <c r="D3" t="n">
-        <v>2.47</v>
+        <v>2.48</v>
       </c>
       <c r="E3" t="n">
         <v>83317</v>
@@ -702,10 +702,10 @@
         <v>55.85</v>
       </c>
       <c r="G3" t="n">
-        <v>37.16</v>
+        <v>37.12</v>
       </c>
       <c r="H3" t="n">
-        <v>2947336650</v>
+        <v>2943898950</v>
       </c>
       <c r="I3" t="n">
         <v>10270</v>
@@ -723,7 +723,7 @@
         <v>-0.42</v>
       </c>
       <c r="N3" t="n">
-        <v>35.77</v>
+        <v>35.73</v>
       </c>
       <c r="O3" t="n">
         <v>91.87</v>
@@ -782,10 +782,10 @@
         <v>2024</v>
       </c>
       <c r="B4" t="n">
-        <v>51.01</v>
+        <v>50.96</v>
       </c>
       <c r="C4" t="n">
-        <v>51.03</v>
+        <v>50.97</v>
       </c>
       <c r="D4" t="n">
         <v>1.96</v>
@@ -797,10 +797,10 @@
         <v>48.85</v>
       </c>
       <c r="G4" t="n">
-        <v>35.32</v>
+        <v>35.28</v>
       </c>
       <c r="H4" t="n">
-        <v>1518188100</v>
+        <v>1516459800</v>
       </c>
       <c r="I4" t="n">
         <v>11056</v>
@@ -818,7 +818,7 @@
         <v>-0.35</v>
       </c>
       <c r="N4" t="n">
-        <v>44.46</v>
+        <v>44.41</v>
       </c>
       <c r="O4" t="n">
         <v>69.23999999999999</v>
@@ -877,10 +877,10 @@
         <v>2023</v>
       </c>
       <c r="B5" t="n">
-        <v>111.14</v>
+        <v>110.97</v>
       </c>
       <c r="C5" t="n">
-        <v>110.91</v>
+        <v>110.74</v>
       </c>
       <c r="D5" t="n">
         <v>0.9</v>
@@ -892,10 +892,10 @@
         <v>16.19</v>
       </c>
       <c r="G5" t="n">
-        <v>21.96</v>
+        <v>21.92</v>
       </c>
       <c r="H5" t="n">
-        <v>485462399.9999999</v>
+        <v>484716299.9999999</v>
       </c>
       <c r="I5" t="n">
         <v>12031</v>
@@ -913,7 +913,7 @@
         <v>-0.06</v>
       </c>
       <c r="N5" t="n">
-        <v>84.38</v>
+        <v>84.25</v>
       </c>
       <c r="O5" t="n">
         <v>19.76</v>
@@ -972,10 +972,10 @@
         <v>2022</v>
       </c>
       <c r="B6" t="n">
-        <v>62.55</v>
+        <v>62.48</v>
       </c>
       <c r="C6" t="n">
-        <v>62.51</v>
+        <v>62.43</v>
       </c>
       <c r="D6" t="n">
         <v>1.6</v>
@@ -987,10 +987,10 @@
         <v>36.23</v>
       </c>
       <c r="G6" t="n">
-        <v>22.93</v>
+        <v>22.9</v>
       </c>
       <c r="H6" t="n">
-        <v>610022400</v>
+        <v>609273600</v>
       </c>
       <c r="I6" t="n">
         <v>11831</v>
@@ -1008,7 +1008,7 @@
         <v>-0.35</v>
       </c>
       <c r="N6" t="n">
-        <v>55.23</v>
+        <v>55.16</v>
       </c>
       <c r="O6" t="n">
         <v>36.65</v>
@@ -1067,10 +1067,10 @@
         <v>2021</v>
       </c>
       <c r="B7" t="n">
-        <v>73.78</v>
+        <v>73.72</v>
       </c>
       <c r="C7" t="n">
-        <v>73.79000000000001</v>
+        <v>73.73</v>
       </c>
       <c r="D7" t="n">
         <v>1.36</v>
@@ -1082,10 +1082,10 @@
         <v>25.98</v>
       </c>
       <c r="G7" t="n">
-        <v>18.92</v>
+        <v>18.9</v>
       </c>
       <c r="H7" t="n">
-        <v>319606000</v>
+        <v>319359200</v>
       </c>
       <c r="I7" t="n">
         <v>7718</v>
@@ -1103,7 +1103,7 @@
         <v>-0.23</v>
       </c>
       <c r="N7" t="n">
-        <v>57.45</v>
+        <v>57.41</v>
       </c>
       <c r="O7" t="n">
         <v>25.64</v>
@@ -1352,13 +1352,13 @@
         <v>2018</v>
       </c>
       <c r="B10" t="n">
-        <v>47.81</v>
+        <v>47.73</v>
       </c>
       <c r="C10" t="n">
-        <v>47.78</v>
+        <v>47.7</v>
       </c>
       <c r="D10" t="n">
-        <v>2.09</v>
+        <v>2.1</v>
       </c>
       <c r="E10" t="n">
         <v>3409</v>
@@ -1367,10 +1367,10 @@
         <v>31.37</v>
       </c>
       <c r="G10" t="n">
-        <v>19.5</v>
+        <v>19.47</v>
       </c>
       <c r="H10" t="n">
-        <v>145676800</v>
+        <v>145437200</v>
       </c>
       <c r="I10" t="n">
         <v>1985</v>
@@ -1388,7 +1388,7 @@
         <v>-0.6899999999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>44.24</v>
+        <v>44.17</v>
       </c>
       <c r="O10" t="n">
         <v>40.78</v>
@@ -1548,7 +1548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1705,1424 +1705,1424 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46138</v>
+        <v>46229</v>
       </c>
       <c r="B2" t="n">
-        <v>83.09999999999999</v>
+        <v>81.36</v>
       </c>
       <c r="C2" t="n">
-        <v>35.89</v>
+        <v>27.65</v>
       </c>
       <c r="D2" t="n">
-        <v>2.79</v>
+        <v>3.62</v>
       </c>
       <c r="E2" t="n">
-        <v>54533</v>
+        <v>64861</v>
       </c>
       <c r="F2" t="n">
-        <v>71.45999999999999</v>
+        <v>62.03</v>
       </c>
       <c r="G2" t="n">
-        <v>24.79</v>
+        <v>21.2</v>
       </c>
       <c r="H2" t="n">
-        <v>4846757020</v>
+        <v>4856142500</v>
       </c>
       <c r="I2" t="n">
-        <v>12814</v>
+        <v>38860</v>
       </c>
       <c r="J2" t="n">
-        <v>80572</v>
+        <v>99369</v>
       </c>
       <c r="K2" t="n">
-        <v>-67758</v>
+        <v>-60509</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.47</v>
+        <v>-0.33</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.35</v>
+        <v>-0.26</v>
       </c>
       <c r="N2" t="n">
-        <v>34.45</v>
+        <v>26.54</v>
       </c>
       <c r="O2" t="n">
-        <v>69.28</v>
+        <v>77.01000000000001</v>
       </c>
       <c r="P2" t="n">
-        <v>54.78</v>
+        <v>55.07</v>
       </c>
       <c r="Q2" t="n">
-        <v>50344</v>
+        <v>24077</v>
       </c>
       <c r="R2" t="n">
-        <v>-26429</v>
+        <v>-8695</v>
       </c>
       <c r="S2" t="n">
-        <v>-21283</v>
+        <v>-6176</v>
       </c>
       <c r="T2" t="n">
-        <v>48587</v>
+        <v>21400</v>
       </c>
       <c r="U2" t="n">
-        <v>1757</v>
+        <v>2677</v>
       </c>
       <c r="V2" t="n">
-        <v>3487</v>
+        <v>4421</v>
       </c>
       <c r="W2" t="n">
-        <v>6321</v>
+        <v>7054</v>
       </c>
       <c r="X2" t="n">
-        <v>22793</v>
+        <v>26792</v>
       </c>
       <c r="Y2" t="n">
-        <v>107111</v>
+        <v>154393</v>
       </c>
       <c r="Z2" t="n">
-        <v>15.48</v>
+        <v>39.39</v>
       </c>
       <c r="AA2" t="n">
-        <v>137069</v>
+        <v>165506</v>
       </c>
       <c r="AB2" t="n">
-        <v>118131</v>
+        <v>115953</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.01</v>
+        <v>0.25</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.42</v>
+        <v>10.13</v>
       </c>
       <c r="AE2" t="n">
-        <v>19312</v>
+        <v>19732</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45956</v>
+        <v>46138</v>
       </c>
       <c r="B3" t="n">
-        <v>154.36</v>
+        <v>83.01000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>51.26</v>
+        <v>35.85</v>
       </c>
       <c r="D3" t="n">
-        <v>1.95</v>
+        <v>2.79</v>
       </c>
       <c r="E3" t="n">
-        <v>36761</v>
+        <v>54533</v>
       </c>
       <c r="F3" t="n">
-        <v>55.98</v>
+        <v>71.45999999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>41.4</v>
+        <v>24.76</v>
       </c>
       <c r="H3" t="n">
-        <v>4925487690</v>
+        <v>4841171240</v>
       </c>
       <c r="I3" t="n">
-        <v>10822</v>
+        <v>12814</v>
       </c>
       <c r="J3" t="n">
-        <v>60608</v>
+        <v>80572</v>
       </c>
       <c r="K3" t="n">
-        <v>-49786</v>
+        <v>-67758</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.45</v>
+        <v>-0.47</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.42</v>
+        <v>-0.35</v>
       </c>
       <c r="N3" t="n">
-        <v>45.04</v>
+        <v>34.41</v>
       </c>
       <c r="O3" t="n">
-        <v>81.09</v>
+        <v>69.28</v>
       </c>
       <c r="P3" t="n">
-        <v>70.16</v>
+        <v>54.78</v>
       </c>
       <c r="Q3" t="n">
-        <v>23751</v>
+        <v>50344</v>
       </c>
       <c r="R3" t="n">
-        <v>-9024</v>
+        <v>-26429</v>
       </c>
       <c r="S3" t="n">
-        <v>-14880</v>
+        <v>-21283</v>
       </c>
       <c r="T3" t="n">
-        <v>22115</v>
+        <v>48587</v>
       </c>
       <c r="U3" t="n">
-        <v>1636</v>
+        <v>1757</v>
       </c>
       <c r="V3" t="n">
-        <v>3062</v>
+        <v>3487</v>
       </c>
       <c r="W3" t="n">
-        <v>4705</v>
+        <v>6321</v>
       </c>
       <c r="X3" t="n">
-        <v>19437</v>
+        <v>22793</v>
       </c>
       <c r="Y3" t="n">
-        <v>90417</v>
+        <v>107111</v>
       </c>
       <c r="Z3" t="n">
-        <v>31.39</v>
+        <v>15.48</v>
       </c>
       <c r="AA3" t="n">
-        <v>84223</v>
+        <v>137069</v>
       </c>
       <c r="AB3" t="n">
-        <v>78615</v>
+        <v>118131</v>
       </c>
       <c r="AC3" t="n">
         <v>0.01</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.76</v>
+        <v>0.42</v>
       </c>
       <c r="AE3" t="n">
-        <v>12456</v>
+        <v>19312</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45865</v>
+        <v>45956</v>
       </c>
       <c r="B4" t="n">
-        <v>164</v>
+        <v>154.17</v>
       </c>
       <c r="C4" t="n">
-        <v>53.57</v>
+        <v>51.2</v>
       </c>
       <c r="D4" t="n">
-        <v>1.87</v>
+        <v>1.95</v>
       </c>
       <c r="E4" t="n">
-        <v>29109</v>
+        <v>36761</v>
       </c>
       <c r="F4" t="n">
-        <v>56.53</v>
+        <v>55.98</v>
       </c>
       <c r="G4" t="n">
-        <v>43.27</v>
+        <v>41.36</v>
       </c>
       <c r="H4" t="n">
-        <v>4333249440</v>
+        <v>4919649210</v>
       </c>
       <c r="I4" t="n">
-        <v>10598</v>
+        <v>10822</v>
       </c>
       <c r="J4" t="n">
-        <v>56791</v>
+        <v>60608</v>
       </c>
       <c r="K4" t="n">
-        <v>-46193</v>
+        <v>-49786</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.5</v>
+        <v>-0.45</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.46</v>
+        <v>-0.42</v>
       </c>
       <c r="N4" t="n">
-        <v>47.2</v>
+        <v>44.99</v>
       </c>
       <c r="O4" t="n">
-        <v>81</v>
+        <v>81.09</v>
       </c>
       <c r="P4" t="n">
-        <v>69.58</v>
+        <v>70.16</v>
       </c>
       <c r="Q4" t="n">
-        <v>15365</v>
+        <v>23751</v>
       </c>
       <c r="R4" t="n">
-        <v>-7127</v>
+        <v>-9024</v>
       </c>
       <c r="S4" t="n">
-        <v>-11833</v>
+        <v>-14880</v>
       </c>
       <c r="T4" t="n">
-        <v>13470</v>
+        <v>22115</v>
       </c>
       <c r="U4" t="n">
-        <v>1895</v>
+        <v>1636</v>
       </c>
       <c r="V4" t="n">
-        <v>2721</v>
+        <v>3062</v>
       </c>
       <c r="W4" t="n">
-        <v>4291</v>
+        <v>4705</v>
       </c>
       <c r="X4" t="n">
-        <v>17481</v>
+        <v>19437</v>
       </c>
       <c r="Y4" t="n">
-        <v>77962</v>
+        <v>90417</v>
       </c>
       <c r="Z4" t="n">
-        <v>36.97</v>
+        <v>31.39</v>
       </c>
       <c r="AA4" t="n">
-        <v>66129</v>
+        <v>84223</v>
       </c>
       <c r="AB4" t="n">
-        <v>62975</v>
+        <v>78615</v>
       </c>
       <c r="AC4" t="n">
         <v>0.01</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.92</v>
+        <v>0.76</v>
       </c>
       <c r="AE4" t="n">
-        <v>9720</v>
+        <v>12456</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45774</v>
+        <v>45865</v>
       </c>
       <c r="B5" t="n">
-        <v>141.75</v>
+        <v>163.81</v>
       </c>
       <c r="C5" t="n">
-        <v>13.15</v>
+        <v>53.5</v>
       </c>
       <c r="D5" t="n">
-        <v>7.6</v>
+        <v>1.87</v>
       </c>
       <c r="E5" t="n">
-        <v>22249</v>
+        <v>29109</v>
       </c>
       <c r="F5" t="n">
-        <v>42.61</v>
+        <v>56.53</v>
       </c>
       <c r="G5" t="n">
-        <v>31.75</v>
+        <v>43.22</v>
       </c>
       <c r="H5" t="n">
-        <v>2661380490</v>
+        <v>4328132580</v>
       </c>
       <c r="I5" t="n">
-        <v>10285</v>
+        <v>10598</v>
       </c>
       <c r="J5" t="n">
-        <v>53691</v>
+        <v>56791</v>
       </c>
       <c r="K5" t="n">
-        <v>-43406</v>
+        <v>-46193</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.54</v>
+        <v>-0.5</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.52</v>
+        <v>-0.46</v>
       </c>
       <c r="N5" t="n">
-        <v>33.4</v>
+        <v>47.15</v>
       </c>
       <c r="O5" t="n">
-        <v>82.97</v>
+        <v>81</v>
       </c>
       <c r="P5" t="n">
-        <v>72.14</v>
+        <v>69.58</v>
       </c>
       <c r="Q5" t="n">
-        <v>27414</v>
+        <v>15365</v>
       </c>
       <c r="R5" t="n">
-        <v>-5216</v>
+        <v>-7127</v>
       </c>
       <c r="S5" t="n">
-        <v>-15553</v>
+        <v>-11833</v>
       </c>
       <c r="T5" t="n">
-        <v>26187</v>
+        <v>13470</v>
       </c>
       <c r="U5" t="n">
-        <v>1227</v>
+        <v>1895</v>
       </c>
       <c r="V5" t="n">
-        <v>1454</v>
+        <v>2721</v>
       </c>
       <c r="W5" t="n">
-        <v>3989</v>
+        <v>4291</v>
       </c>
       <c r="X5" t="n">
-        <v>14643</v>
+        <v>17481</v>
       </c>
       <c r="Y5" t="n">
-        <v>63393</v>
+        <v>77962</v>
       </c>
       <c r="Z5" t="n">
-        <v>12.03</v>
+        <v>36.97</v>
       </c>
       <c r="AA5" t="n">
-        <v>73337</v>
+        <v>66129</v>
       </c>
       <c r="AB5" t="n">
-        <v>72769</v>
+        <v>62975</v>
       </c>
       <c r="AC5" t="n">
         <v>0.01</v>
       </c>
       <c r="AD5" t="n">
-        <v>1.3</v>
+        <v>0.92</v>
       </c>
       <c r="AE5" t="n">
-        <v>14095</v>
+        <v>9720</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45592</v>
+        <v>45774</v>
       </c>
       <c r="B6" t="n">
-        <v>168.61</v>
+        <v>141.6</v>
       </c>
       <c r="C6" t="n">
-        <v>11.79</v>
+        <v>13.14</v>
       </c>
       <c r="D6" t="n">
-        <v>8.48</v>
+        <v>7.61</v>
       </c>
       <c r="E6" t="n">
-        <v>22347</v>
+        <v>22249</v>
       </c>
       <c r="F6" t="n">
-        <v>55.04</v>
+        <v>42.61</v>
       </c>
       <c r="G6" t="n">
-        <v>49.33</v>
+        <v>31.71</v>
       </c>
       <c r="H6" t="n">
-        <v>3255774430</v>
+        <v>2658447570</v>
       </c>
       <c r="I6" t="n">
-        <v>10225</v>
+        <v>10285</v>
       </c>
       <c r="J6" t="n">
-        <v>38487</v>
+        <v>53691</v>
       </c>
       <c r="K6" t="n">
-        <v>-28262</v>
+        <v>-43406</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.41</v>
+        <v>-0.54</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.43</v>
+        <v>-0.52</v>
       </c>
       <c r="N6" t="n">
-        <v>47.23</v>
+        <v>33.36</v>
       </c>
       <c r="O6" t="n">
-        <v>91.09999999999999</v>
+        <v>82.97</v>
       </c>
       <c r="P6" t="n">
-        <v>76.90000000000001</v>
+        <v>72.14</v>
       </c>
       <c r="Q6" t="n">
-        <v>17627</v>
+        <v>27414</v>
       </c>
       <c r="R6" t="n">
-        <v>-4346</v>
+        <v>-5216</v>
       </c>
       <c r="S6" t="n">
-        <v>-12745</v>
+        <v>-15553</v>
       </c>
       <c r="T6" t="n">
-        <v>16814</v>
+        <v>26187</v>
       </c>
       <c r="U6" t="n">
-        <v>813</v>
+        <v>1227</v>
       </c>
       <c r="V6" t="n">
-        <v>744</v>
+        <v>1454</v>
       </c>
       <c r="W6" t="n">
-        <v>3390</v>
+        <v>3989</v>
       </c>
       <c r="X6" t="n">
-        <v>12238</v>
+        <v>14643</v>
       </c>
       <c r="Y6" t="n">
-        <v>51161</v>
+        <v>63393</v>
       </c>
       <c r="Z6" t="n">
-        <v>26.54</v>
+        <v>12.03</v>
       </c>
       <c r="AA6" t="n">
-        <v>54741</v>
+        <v>73337</v>
       </c>
       <c r="AB6" t="n">
-        <v>54655</v>
+        <v>72769</v>
       </c>
       <c r="AC6" t="n">
         <v>0.01</v>
       </c>
       <c r="AD6" t="n">
-        <v>1.27</v>
+        <v>1.3</v>
       </c>
       <c r="AE6" t="n">
-        <v>10997</v>
+        <v>14095</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45501</v>
+        <v>45592</v>
       </c>
       <c r="B7" t="n">
-        <v>173.18</v>
+        <v>168.41</v>
       </c>
       <c r="C7" t="n">
-        <v>9.02</v>
+        <v>11.77</v>
       </c>
       <c r="D7" t="n">
-        <v>11.09</v>
+        <v>8.49</v>
       </c>
       <c r="E7" t="n">
-        <v>19075</v>
+        <v>22347</v>
       </c>
       <c r="F7" t="n">
-        <v>55.26</v>
+        <v>55.04</v>
       </c>
       <c r="G7" t="n">
-        <v>49.35</v>
+        <v>49.28</v>
       </c>
       <c r="H7" t="n">
-        <v>2874642880</v>
+        <v>3251849150</v>
       </c>
       <c r="I7" t="n">
-        <v>10015</v>
+        <v>10225</v>
       </c>
       <c r="J7" t="n">
-        <v>34800</v>
+        <v>38487</v>
       </c>
       <c r="K7" t="n">
-        <v>-24785</v>
+        <v>-28262</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.46</v>
+        <v>-0.41</v>
       </c>
       <c r="M7" t="n">
         <v>-0.43</v>
       </c>
       <c r="N7" t="n">
-        <v>53.35</v>
+        <v>47.18</v>
       </c>
       <c r="O7" t="n">
-        <v>80.66</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="P7" t="n">
-        <v>67.01000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="Q7" t="n">
-        <v>14488</v>
+        <v>17627</v>
       </c>
       <c r="R7" t="n">
-        <v>-3184</v>
+        <v>-4346</v>
       </c>
       <c r="S7" t="n">
-        <v>-10320</v>
+        <v>-12745</v>
       </c>
       <c r="T7" t="n">
-        <v>13511</v>
+        <v>16814</v>
       </c>
       <c r="U7" t="n">
-        <v>977</v>
+        <v>813</v>
       </c>
       <c r="V7" t="n">
-        <v>333</v>
+        <v>744</v>
       </c>
       <c r="W7" t="n">
-        <v>3090</v>
+        <v>3390</v>
       </c>
       <c r="X7" t="n">
-        <v>10477</v>
+        <v>12238</v>
       </c>
       <c r="Y7" t="n">
-        <v>45664</v>
+        <v>51161</v>
       </c>
       <c r="Z7" t="n">
-        <v>30.29</v>
+        <v>26.54</v>
       </c>
       <c r="AA7" t="n">
-        <v>40719</v>
+        <v>54741</v>
       </c>
       <c r="AB7" t="n">
-        <v>41894</v>
+        <v>54655</v>
       </c>
       <c r="AC7" t="n">
         <v>0.01</v>
       </c>
       <c r="AD7" t="n">
-        <v>1.48</v>
+        <v>1.27</v>
       </c>
       <c r="AE7" t="n">
-        <v>7158</v>
+        <v>10997</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45410</v>
+        <v>45501</v>
       </c>
       <c r="B8" t="n">
-        <v>142.86</v>
+        <v>172.99</v>
       </c>
       <c r="C8" t="n">
-        <v>65.81999999999999</v>
+        <v>9.01</v>
       </c>
       <c r="D8" t="n">
-        <v>1.52</v>
+        <v>11.1</v>
       </c>
       <c r="E8" t="n">
-        <v>17319</v>
+        <v>19075</v>
       </c>
       <c r="F8" t="n">
-        <v>57.14</v>
+        <v>55.26</v>
       </c>
       <c r="G8" t="n">
-        <v>43.26</v>
+        <v>49.3</v>
       </c>
       <c r="H8" t="n">
-        <v>2125937000</v>
+        <v>2871447740</v>
       </c>
       <c r="I8" t="n">
-        <v>11237</v>
+        <v>10015</v>
       </c>
       <c r="J8" t="n">
-        <v>31438</v>
+        <v>34800</v>
       </c>
       <c r="K8" t="n">
-        <v>-20201</v>
+        <v>-24785</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.53</v>
+        <v>-0.46</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.41</v>
+        <v>-0.43</v>
       </c>
       <c r="N8" t="n">
-        <v>56.78</v>
+        <v>53.29</v>
       </c>
       <c r="O8" t="n">
-        <v>65.84</v>
+        <v>80.66</v>
       </c>
       <c r="P8" t="n">
-        <v>52.39</v>
+        <v>67.01000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>15345</v>
+        <v>14488</v>
       </c>
       <c r="R8" t="n">
-        <v>-5693</v>
+        <v>-3184</v>
       </c>
       <c r="S8" t="n">
-        <v>-9345</v>
+        <v>-10320</v>
       </c>
       <c r="T8" t="n">
-        <v>14976</v>
+        <v>13511</v>
       </c>
       <c r="U8" t="n">
-        <v>369</v>
+        <v>977</v>
       </c>
       <c r="V8" t="n">
-        <v>-347</v>
+        <v>333</v>
       </c>
       <c r="W8" t="n">
-        <v>2720</v>
+        <v>3090</v>
       </c>
       <c r="X8" t="n">
-        <v>8582</v>
+        <v>10477</v>
       </c>
       <c r="Y8" t="n">
-        <v>38506</v>
+        <v>45664</v>
       </c>
       <c r="Z8" t="n">
-        <v>29.48</v>
+        <v>30.29</v>
       </c>
       <c r="AA8" t="n">
-        <v>30709</v>
+        <v>40719</v>
       </c>
       <c r="AB8" t="n">
-        <v>30837</v>
+        <v>41894</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.66</v>
+        <v>1.48</v>
       </c>
       <c r="AE8" t="n">
-        <v>7740</v>
+        <v>7158</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45228</v>
+        <v>45410</v>
       </c>
       <c r="B9" t="n">
-        <v>108.81</v>
+        <v>142.7</v>
       </c>
       <c r="C9" t="n">
-        <v>55.44</v>
+        <v>65.73999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>1.8</v>
+        <v>1.52</v>
       </c>
       <c r="E9" t="n">
-        <v>10789</v>
+        <v>17319</v>
       </c>
       <c r="F9" t="n">
-        <v>51.01</v>
+        <v>57.14</v>
       </c>
       <c r="G9" t="n">
-        <v>30.23</v>
+        <v>43.21</v>
       </c>
       <c r="H9" t="n">
-        <v>1005710000</v>
+        <v>2123475000</v>
       </c>
       <c r="I9" t="n">
-        <v>11027</v>
+        <v>11237</v>
       </c>
       <c r="J9" t="n">
-        <v>18281</v>
+        <v>31438</v>
       </c>
       <c r="K9" t="n">
-        <v>-7254</v>
+        <v>-20201</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.34</v>
+        <v>-0.53</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.22</v>
+        <v>-0.41</v>
       </c>
       <c r="N9" t="n">
-        <v>47.15</v>
+        <v>56.72</v>
       </c>
       <c r="O9" t="n">
-        <v>54.57</v>
+        <v>65.84</v>
       </c>
       <c r="P9" t="n">
-        <v>40.16</v>
+        <v>52.39</v>
       </c>
       <c r="Q9" t="n">
-        <v>7332</v>
+        <v>15345</v>
       </c>
       <c r="R9" t="n">
-        <v>-3170</v>
+        <v>-5693</v>
       </c>
       <c r="S9" t="n">
-        <v>-4525</v>
+        <v>-9345</v>
       </c>
       <c r="T9" t="n">
-        <v>7054</v>
+        <v>14976</v>
       </c>
       <c r="U9" t="n">
-        <v>278</v>
+        <v>369</v>
       </c>
       <c r="V9" t="n">
-        <v>-182</v>
+        <v>-347</v>
       </c>
       <c r="W9" t="n">
-        <v>2294</v>
+        <v>2720</v>
       </c>
       <c r="X9" t="n">
-        <v>7972</v>
+        <v>8582</v>
       </c>
       <c r="Y9" t="n">
-        <v>23557</v>
+        <v>38506</v>
       </c>
       <c r="Z9" t="n">
-        <v>63.16</v>
+        <v>29.48</v>
       </c>
       <c r="AA9" t="n">
-        <v>13823</v>
+        <v>30709</v>
       </c>
       <c r="AB9" t="n">
-        <v>14451</v>
+        <v>30837</v>
       </c>
       <c r="AC9" t="n">
         <v>0.04</v>
       </c>
       <c r="AD9" t="n">
-        <v>1.05</v>
+        <v>0.66</v>
       </c>
       <c r="AE9" t="n">
-        <v>3807</v>
+        <v>7740</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45137</v>
+        <v>45228</v>
       </c>
       <c r="B10" t="n">
-        <v>186.59</v>
+        <v>108.67</v>
       </c>
       <c r="C10" t="n">
-        <v>120.96</v>
+        <v>55.37</v>
       </c>
       <c r="D10" t="n">
-        <v>0.83</v>
+        <v>1.81</v>
       </c>
       <c r="E10" t="n">
-        <v>7165</v>
+        <v>10789</v>
       </c>
       <c r="F10" t="n">
-        <v>45.81</v>
+        <v>51.01</v>
       </c>
       <c r="G10" t="n">
-        <v>41.99</v>
+        <v>30.19</v>
       </c>
       <c r="H10" t="n">
-        <v>1154643700</v>
+        <v>1004476000</v>
       </c>
       <c r="I10" t="n">
-        <v>10954</v>
+        <v>11027</v>
       </c>
       <c r="J10" t="n">
-        <v>16023</v>
+        <v>18281</v>
       </c>
       <c r="K10" t="n">
-        <v>-5069</v>
+        <v>-7254</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.44</v>
+        <v>-0.34</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.18</v>
+        <v>-0.22</v>
       </c>
       <c r="N10" t="n">
-        <v>100.21</v>
+        <v>47.09</v>
       </c>
       <c r="O10" t="n">
-        <v>34.79</v>
+        <v>54.57</v>
       </c>
       <c r="P10" t="n">
-        <v>24.26</v>
+        <v>40.16</v>
       </c>
       <c r="Q10" t="n">
-        <v>6348</v>
+        <v>7332</v>
       </c>
       <c r="R10" t="n">
-        <v>-446</v>
+        <v>-3170</v>
       </c>
       <c r="S10" t="n">
-        <v>-5099</v>
+        <v>-4525</v>
       </c>
       <c r="T10" t="n">
-        <v>6059</v>
+        <v>7054</v>
       </c>
       <c r="U10" t="n">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="V10" t="n">
-        <v>-33</v>
+        <v>-182</v>
       </c>
       <c r="W10" t="n">
-        <v>2040</v>
+        <v>2294</v>
       </c>
       <c r="X10" t="n">
-        <v>7651</v>
+        <v>7972</v>
       </c>
       <c r="Y10" t="n">
-        <v>18463</v>
+        <v>23557</v>
       </c>
       <c r="Z10" t="n">
-        <v>91.86999999999999</v>
+        <v>63.16</v>
       </c>
       <c r="AA10" t="n">
-        <v>7430</v>
+        <v>13823</v>
       </c>
       <c r="AB10" t="n">
-        <v>8013</v>
+        <v>14451</v>
       </c>
       <c r="AC10" t="n">
         <v>0.04</v>
       </c>
       <c r="AD10" t="n">
-        <v>1.62</v>
+        <v>1.05</v>
       </c>
       <c r="AE10" t="n">
-        <v>3067</v>
+        <v>3807</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45046</v>
+        <v>45137</v>
       </c>
       <c r="B11" t="n">
-        <v>335.14</v>
+        <v>186.39</v>
       </c>
       <c r="C11" t="n">
-        <v>137.91</v>
+        <v>120.83</v>
       </c>
       <c r="D11" t="n">
-        <v>0.73</v>
+        <v>0.83</v>
       </c>
       <c r="E11" t="n">
-        <v>2524</v>
+        <v>7165</v>
       </c>
       <c r="F11" t="n">
-        <v>28.41</v>
+        <v>45.81</v>
       </c>
       <c r="G11" t="n">
-        <v>27.92</v>
+        <v>41.94</v>
       </c>
       <c r="H11" t="n">
-        <v>684684000</v>
+        <v>1153407200</v>
       </c>
       <c r="I11" t="n">
-        <v>12080</v>
+        <v>10954</v>
       </c>
       <c r="J11" t="n">
-        <v>15320</v>
+        <v>16023</v>
       </c>
       <c r="K11" t="n">
-        <v>-3240</v>
+        <v>-5069</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.49</v>
+        <v>-0.44</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.13</v>
+        <v>-0.18</v>
       </c>
       <c r="N11" t="n">
-        <v>104.07</v>
+        <v>100.1</v>
       </c>
       <c r="O11" t="n">
-        <v>20.38</v>
+        <v>34.79</v>
       </c>
       <c r="P11" t="n">
-        <v>13.67</v>
+        <v>24.26</v>
       </c>
       <c r="Q11" t="n">
-        <v>2911</v>
+        <v>6348</v>
       </c>
       <c r="R11" t="n">
-        <v>-841</v>
+        <v>-446</v>
       </c>
       <c r="S11" t="n">
-        <v>-380</v>
+        <v>-5099</v>
       </c>
       <c r="T11" t="n">
-        <v>2663</v>
+        <v>6059</v>
       </c>
       <c r="U11" t="n">
-        <v>248</v>
+        <v>289</v>
       </c>
       <c r="V11" t="n">
-        <v>70</v>
+        <v>-33</v>
       </c>
       <c r="W11" t="n">
-        <v>1875</v>
+        <v>2040</v>
       </c>
       <c r="X11" t="n">
-        <v>7332</v>
+        <v>7651</v>
       </c>
       <c r="Y11" t="n">
-        <v>17623</v>
+        <v>18463</v>
       </c>
       <c r="Z11" t="n">
-        <v>151.17</v>
+        <v>91.86999999999999</v>
       </c>
       <c r="AA11" t="n">
-        <v>4696</v>
+        <v>7430</v>
       </c>
       <c r="AB11" t="n">
-        <v>4423</v>
+        <v>8013</v>
       </c>
       <c r="AC11" t="n">
         <v>0.04</v>
       </c>
       <c r="AD11" t="n">
-        <v>4.85</v>
+        <v>1.62</v>
       </c>
       <c r="AE11" t="n">
-        <v>0</v>
+        <v>3067</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44864</v>
+        <v>45046</v>
       </c>
       <c r="B12" t="n">
-        <v>492.22</v>
+        <v>334.77</v>
       </c>
       <c r="C12" t="n">
-        <v>62.12</v>
+        <v>137.76</v>
       </c>
       <c r="D12" t="n">
-        <v>1.61</v>
+        <v>0.73</v>
       </c>
       <c r="E12" t="n">
-        <v>1007</v>
+        <v>2524</v>
       </c>
       <c r="F12" t="n">
-        <v>11.47</v>
+        <v>28.41</v>
       </c>
       <c r="G12" t="n">
-        <v>15.67</v>
+        <v>27.89</v>
       </c>
       <c r="H12" t="n">
-        <v>334708400</v>
+        <v>683943000.0000001</v>
       </c>
       <c r="I12" t="n">
-        <v>11904</v>
+        <v>12080</v>
       </c>
       <c r="J12" t="n">
-        <v>13143</v>
+        <v>15320</v>
       </c>
       <c r="K12" t="n">
-        <v>-1239</v>
+        <v>-3240</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.18</v>
+        <v>-0.49</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.06</v>
+        <v>-0.13</v>
       </c>
       <c r="N12" t="n">
-        <v>47.62</v>
+        <v>103.96</v>
       </c>
       <c r="O12" t="n">
-        <v>25.38</v>
+        <v>20.38</v>
       </c>
       <c r="P12" t="n">
-        <v>16.62</v>
+        <v>13.67</v>
       </c>
       <c r="Q12" t="n">
-        <v>392</v>
+        <v>2911</v>
       </c>
       <c r="R12" t="n">
-        <v>3148</v>
+        <v>-841</v>
       </c>
       <c r="S12" t="n">
-        <v>-3753</v>
+        <v>-380</v>
       </c>
       <c r="T12" t="n">
-        <v>-138</v>
+        <v>2663</v>
       </c>
       <c r="U12" t="n">
-        <v>530</v>
+        <v>248</v>
       </c>
       <c r="V12" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="W12" t="n">
-        <v>1945</v>
+        <v>1875</v>
       </c>
       <c r="X12" t="n">
-        <v>6920</v>
+        <v>7332</v>
       </c>
       <c r="Y12" t="n">
-        <v>16368</v>
+        <v>17623</v>
       </c>
       <c r="Z12" t="n">
-        <v>150.65</v>
+        <v>151.17</v>
       </c>
       <c r="AA12" t="n">
-        <v>2875</v>
+        <v>4696</v>
       </c>
       <c r="AB12" t="n">
-        <v>4104</v>
+        <v>4423</v>
       </c>
       <c r="AC12" t="n">
         <v>0.04</v>
       </c>
       <c r="AD12" t="n">
-        <v>14.71</v>
+        <v>4.85</v>
       </c>
       <c r="AE12" t="n">
-        <v>3485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44773</v>
+        <v>44864</v>
       </c>
       <c r="B13" t="n">
-        <v>689.55</v>
+        <v>491.49</v>
       </c>
       <c r="C13" t="n">
-        <v>63.61</v>
+        <v>62.03</v>
       </c>
       <c r="D13" t="n">
-        <v>1.57</v>
+        <v>1.61</v>
       </c>
       <c r="E13" t="n">
-        <v>877</v>
+        <v>1007</v>
       </c>
       <c r="F13" t="n">
-        <v>9.789999999999999</v>
+        <v>11.47</v>
       </c>
       <c r="G13" t="n">
-        <v>18.96</v>
+        <v>15.65</v>
       </c>
       <c r="H13" t="n">
-        <v>452343499.9999999</v>
+        <v>334211800.0000001</v>
       </c>
       <c r="I13" t="n">
-        <v>11837</v>
+        <v>11904</v>
       </c>
       <c r="J13" t="n">
-        <v>17037</v>
+        <v>13143</v>
       </c>
       <c r="K13" t="n">
-        <v>-5200</v>
+        <v>-1239</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.59</v>
+        <v>-0.18</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.22</v>
+        <v>-0.06</v>
       </c>
       <c r="N13" t="n">
-        <v>52.12</v>
+        <v>47.55</v>
       </c>
       <c r="O13" t="n">
-        <v>29.82</v>
+        <v>25.38</v>
       </c>
       <c r="P13" t="n">
-        <v>20.4</v>
+        <v>16.62</v>
       </c>
       <c r="Q13" t="n">
-        <v>1270</v>
+        <v>392</v>
       </c>
       <c r="R13" t="n">
-        <v>1618</v>
+        <v>3148</v>
       </c>
       <c r="S13" t="n">
-        <v>-3762</v>
+        <v>-3753</v>
       </c>
       <c r="T13" t="n">
-        <v>837</v>
+        <v>-138</v>
       </c>
       <c r="U13" t="n">
-        <v>433</v>
+        <v>530</v>
       </c>
       <c r="V13" t="n">
-        <v>-97</v>
+        <v>130</v>
       </c>
       <c r="W13" t="n">
-        <v>1824</v>
+        <v>1945</v>
       </c>
       <c r="X13" t="n">
-        <v>5993</v>
+        <v>6920</v>
       </c>
       <c r="Y13" t="n">
-        <v>19845</v>
+        <v>16368</v>
       </c>
       <c r="Z13" t="n">
-        <v>87.98</v>
+        <v>150.65</v>
       </c>
       <c r="AA13" t="n">
-        <v>10772</v>
+        <v>2875</v>
       </c>
       <c r="AB13" t="n">
-        <v>7165</v>
+        <v>4104</v>
       </c>
       <c r="AC13" t="n">
         <v>0.04</v>
       </c>
       <c r="AD13" t="n">
-        <v>15.24</v>
+        <v>14.71</v>
       </c>
       <c r="AE13" t="n">
-        <v>3345</v>
+        <v>3485</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44652</v>
+        <v>44773</v>
       </c>
       <c r="B14" t="n">
-        <v>286.69</v>
+        <v>688.79</v>
       </c>
       <c r="C14" t="n">
-        <v>32.65</v>
+        <v>63.54</v>
       </c>
       <c r="D14" t="n">
-        <v>3.06</v>
+        <v>1.57</v>
       </c>
       <c r="E14" t="n">
-        <v>2202</v>
+        <v>877</v>
       </c>
       <c r="F14" t="n">
-        <v>19.52</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>17.63</v>
+        <v>18.94</v>
       </c>
       <c r="H14" t="n">
-        <v>463860600.0000001</v>
+        <v>451844500</v>
       </c>
       <c r="I14" t="n">
-        <v>11846</v>
+        <v>11837</v>
       </c>
       <c r="J14" t="n">
-        <v>20338</v>
+        <v>17037</v>
       </c>
       <c r="K14" t="n">
-        <v>-8492</v>
+        <v>-5200</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.84</v>
+        <v>-0.59</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.32</v>
+        <v>-0.22</v>
       </c>
       <c r="N14" t="n">
-        <v>46.59</v>
+        <v>52.07</v>
       </c>
       <c r="O14" t="n">
-        <v>31.79</v>
+        <v>29.82</v>
       </c>
       <c r="P14" t="n">
-        <v>22.08</v>
+        <v>20.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>1731</v>
+        <v>1270</v>
       </c>
       <c r="R14" t="n">
-        <v>2612</v>
+        <v>1618</v>
       </c>
       <c r="S14" t="n">
-        <v>-2446</v>
+        <v>-3762</v>
       </c>
       <c r="T14" t="n">
-        <v>1370</v>
+        <v>837</v>
       </c>
       <c r="U14" t="n">
-        <v>361</v>
+        <v>433</v>
       </c>
       <c r="V14" t="n">
-        <v>-135</v>
+        <v>-97</v>
       </c>
       <c r="W14" t="n">
-        <v>1618</v>
+        <v>1824</v>
       </c>
       <c r="X14" t="n">
-        <v>5284</v>
+        <v>5993</v>
       </c>
       <c r="Y14" t="n">
-        <v>24013</v>
+        <v>19845</v>
       </c>
       <c r="Z14" t="n">
-        <v>88.73</v>
+        <v>87.98</v>
       </c>
       <c r="AA14" t="n">
-        <v>10288</v>
+        <v>10772</v>
       </c>
       <c r="AB14" t="n">
-        <v>5956</v>
+        <v>7165</v>
       </c>
       <c r="AC14" t="n">
         <v>0.04</v>
       </c>
       <c r="AD14" t="n">
-        <v>6.18</v>
+        <v>15.24</v>
       </c>
       <c r="AE14" t="n">
-        <v>1996</v>
+        <v>3345</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44500</v>
+        <v>44652</v>
       </c>
       <c r="B15" t="n">
-        <v>258.72</v>
+        <v>286.38</v>
       </c>
       <c r="C15" t="n">
-        <v>35.53</v>
+        <v>32.61</v>
       </c>
       <c r="D15" t="n">
-        <v>2.81</v>
+        <v>3.07</v>
       </c>
       <c r="E15" t="n">
-        <v>2969</v>
+        <v>2202</v>
       </c>
       <c r="F15" t="n">
-        <v>34.69</v>
+        <v>19.52</v>
       </c>
       <c r="G15" t="n">
-        <v>26.8</v>
+        <v>17.61</v>
       </c>
       <c r="H15" t="n">
-        <v>637494900</v>
+        <v>463359399.9999999</v>
       </c>
       <c r="I15" t="n">
-        <v>11827</v>
+        <v>11846</v>
       </c>
       <c r="J15" t="n">
-        <v>19298</v>
+        <v>20338</v>
       </c>
       <c r="K15" t="n">
-        <v>-7471</v>
+        <v>-8492</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.78</v>
+        <v>-0.84</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.31</v>
+        <v>-0.32</v>
       </c>
       <c r="N15" t="n">
-        <v>66.95</v>
+        <v>46.54</v>
       </c>
       <c r="O15" t="n">
-        <v>33.98</v>
+        <v>31.79</v>
       </c>
       <c r="P15" t="n">
-        <v>22.82</v>
+        <v>22.08</v>
       </c>
       <c r="Q15" t="n">
-        <v>1519</v>
+        <v>1731</v>
       </c>
       <c r="R15" t="n">
-        <v>-4439</v>
+        <v>2612</v>
       </c>
       <c r="S15" t="n">
-        <v>-1420</v>
+        <v>-2446</v>
       </c>
       <c r="T15" t="n">
-        <v>1297</v>
+        <v>1370</v>
       </c>
       <c r="U15" t="n">
-        <v>222</v>
+        <v>361</v>
       </c>
       <c r="V15" t="n">
-        <v>384</v>
+        <v>-135</v>
       </c>
       <c r="W15" t="n">
-        <v>1403</v>
+        <v>1618</v>
       </c>
       <c r="X15" t="n">
-        <v>5232</v>
+        <v>5284</v>
       </c>
       <c r="Y15" t="n">
-        <v>22194</v>
+        <v>24013</v>
       </c>
       <c r="Z15" t="n">
-        <v>86.39</v>
+        <v>88.73</v>
       </c>
       <c r="AA15" t="n">
-        <v>9887</v>
+        <v>10288</v>
       </c>
       <c r="AB15" t="n">
-        <v>5734</v>
+        <v>5956</v>
       </c>
       <c r="AC15" t="n">
         <v>0.04</v>
       </c>
       <c r="AD15" t="n">
-        <v>4.06</v>
+        <v>6.18</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44378</v>
+        <v>44500</v>
       </c>
       <c r="B16" t="n">
-        <v>204.25</v>
+        <v>258.42</v>
       </c>
       <c r="C16" t="n">
-        <v>27.01</v>
+        <v>35.49</v>
       </c>
       <c r="D16" t="n">
-        <v>3.7</v>
+        <v>2.82</v>
       </c>
       <c r="E16" t="n">
-        <v>2730</v>
+        <v>2969</v>
       </c>
       <c r="F16" t="n">
-        <v>36.48</v>
+        <v>34.69</v>
       </c>
       <c r="G16" t="n">
-        <v>22.94</v>
+        <v>26.76</v>
       </c>
       <c r="H16" t="n">
-        <v>484888500</v>
+        <v>636745200.0000001</v>
       </c>
       <c r="I16" t="n">
-        <v>12791</v>
+        <v>11827</v>
       </c>
       <c r="J16" t="n">
-        <v>19654</v>
+        <v>19298</v>
       </c>
       <c r="K16" t="n">
-        <v>-6863</v>
+        <v>-7471</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.89</v>
+        <v>-0.78</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.32</v>
+        <v>-0.31</v>
       </c>
       <c r="N16" t="n">
-        <v>63.71</v>
+        <v>66.88</v>
       </c>
       <c r="O16" t="n">
-        <v>29.53</v>
+        <v>33.98</v>
       </c>
       <c r="P16" t="n">
-        <v>18.56</v>
+        <v>22.82</v>
       </c>
       <c r="Q16" t="n">
-        <v>2682</v>
+        <v>1519</v>
       </c>
       <c r="R16" t="n">
-        <v>-2533</v>
+        <v>-4439</v>
       </c>
       <c r="S16" t="n">
-        <v>4501</v>
+        <v>-1420</v>
       </c>
       <c r="T16" t="n">
-        <v>2499</v>
+        <v>1297</v>
       </c>
       <c r="U16" t="n">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="V16" t="n">
-        <v>56</v>
+        <v>384</v>
       </c>
       <c r="W16" t="n">
-        <v>1245</v>
+        <v>1403</v>
       </c>
       <c r="X16" t="n">
-        <v>4498</v>
+        <v>5232</v>
       </c>
       <c r="Y16" t="n">
-        <v>21358</v>
+        <v>22194</v>
       </c>
       <c r="Z16" t="n">
-        <v>78.73999999999999</v>
+        <v>86.39</v>
       </c>
       <c r="AA16" t="n">
-        <v>10704</v>
+        <v>9887</v>
       </c>
       <c r="AB16" t="n">
-        <v>5878</v>
+        <v>5734</v>
       </c>
       <c r="AC16" t="n">
         <v>0.04</v>
       </c>
       <c r="AD16" t="n">
-        <v>4.17</v>
+        <v>4.06</v>
       </c>
       <c r="AE16" t="n">
         <v>0</v>
@@ -3130,96 +3130,191 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
+        <v>44378</v>
+      </c>
+      <c r="B17" t="n">
+        <v>204.04</v>
+      </c>
+      <c r="C17" t="n">
+        <v>26.99</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2730</v>
+      </c>
+      <c r="F17" t="n">
+        <v>36.48</v>
+      </c>
+      <c r="G17" t="n">
+        <v>22.91</v>
+      </c>
+      <c r="H17" t="n">
+        <v>484389900</v>
+      </c>
+      <c r="I17" t="n">
+        <v>12791</v>
+      </c>
+      <c r="J17" t="n">
+        <v>19654</v>
+      </c>
+      <c r="K17" t="n">
+        <v>-6863</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="N17" t="n">
+        <v>63.64</v>
+      </c>
+      <c r="O17" t="n">
+        <v>29.53</v>
+      </c>
+      <c r="P17" t="n">
+        <v>18.56</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>2682</v>
+      </c>
+      <c r="R17" t="n">
+        <v>-2533</v>
+      </c>
+      <c r="S17" t="n">
+        <v>4501</v>
+      </c>
+      <c r="T17" t="n">
+        <v>2499</v>
+      </c>
+      <c r="U17" t="n">
+        <v>183</v>
+      </c>
+      <c r="V17" t="n">
+        <v>56</v>
+      </c>
+      <c r="W17" t="n">
+        <v>1245</v>
+      </c>
+      <c r="X17" t="n">
+        <v>4498</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>21358</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>78.73999999999999</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>10704</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>5878</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>44288</v>
       </c>
-      <c r="B17" t="n">
-        <v>194.48</v>
-      </c>
-      <c r="C17" t="n">
-        <v>77.36</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="B18" t="n">
+        <v>194.22</v>
+      </c>
+      <c r="C18" t="n">
+        <v>77.26000000000001</v>
+      </c>
+      <c r="D18" t="n">
         <v>1.29</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>2237</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>33.77</v>
       </c>
-      <c r="G17" t="n">
-        <v>19.81</v>
-      </c>
-      <c r="H17" t="n">
-        <v>371854800.0000001</v>
-      </c>
-      <c r="I17" t="n">
+      <c r="G18" t="n">
+        <v>19.78</v>
+      </c>
+      <c r="H18" t="n">
+        <v>371358000</v>
+      </c>
+      <c r="I18" t="n">
         <v>7738</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J18" t="n">
         <v>12667</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K18" t="n">
         <v>-4929</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L18" t="n">
         <v>-0.8100000000000001</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M18" t="n">
         <v>-0.26</v>
       </c>
-      <c r="N17" t="n">
-        <v>62.05</v>
-      </c>
-      <c r="O17" t="n">
+      <c r="N18" t="n">
+        <v>61.97</v>
+      </c>
+      <c r="O18" t="n">
         <v>25.5</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>18.05</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q18" t="n">
         <v>1874</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R18" t="n">
         <v>-1272</v>
       </c>
-      <c r="S17" t="n">
+      <c r="S18" t="n">
         <v>-471</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T18" t="n">
         <v>1576</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U18" t="n">
         <v>298</v>
       </c>
-      <c r="V17" t="n">
+      <c r="V18" t="n">
         <v>52</v>
       </c>
-      <c r="W17" t="n">
+      <c r="W18" t="n">
         <v>1153</v>
       </c>
-      <c r="X17" t="n">
+      <c r="X18" t="n">
         <v>3984</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Y18" t="n">
         <v>14123</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="Z18" t="n">
         <v>96.03</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AA18" t="n">
         <v>9094</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB18" t="n">
         <v>3995</v>
       </c>
-      <c r="AC17" t="n">
+      <c r="AC18" t="n">
         <v>0.16</v>
       </c>
-      <c r="AD17" t="n">
+      <c r="AD18" t="n">
         <v>5.18</v>
       </c>
-      <c r="AE17" t="n">
+      <c r="AE18" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>